<commit_message>
Episode 3: Brian's label review (G-013 now correct)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UnQARerZCp9G2LvKPPit2J
</commit_message>
<xml_diff>
--- a/results/episode-3/labels-review.xlsx
+++ b/results/episode-3/labels-review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/briancorbin/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA3D82A-DFC0-FF40-9E3F-A7C8F5C2CE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2727C770-7F6E-6E43-A29E-7020B02EAC5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="680" windowWidth="34200" windowHeight="21460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Review" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="512">
   <si>
     <t>ID</t>
   </si>
@@ -1755,6 +1755,27 @@
   </si>
   <si>
     <t>the correct answer was ranked higher so seems selection needs adjustment.</t>
+  </si>
+  <si>
+    <t>correct - the question doesn't require the info level to be stated but is improved when it is.</t>
+  </si>
+  <si>
+    <t>The reference answer, however, is noticeably more quantitative as to the motivation.</t>
+  </si>
+  <si>
+    <t>The reference answer arguably provides more detail than the question requires.</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Agreed with note.</t>
+  </si>
+  <si>
+    <t>Completely irrelevant response.</t>
+  </si>
+  <si>
+    <t>Seemed like a bit of a harsh judgement - perhaps review this.</t>
   </si>
 </sst>
 </file>
@@ -1867,7 +1888,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1915,6 +1936,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2189,6 +2213,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:S51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2270,7 +2295,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>19</v>
       </c>
@@ -2323,7 +2348,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>31</v>
       </c>
@@ -2376,7 +2401,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>41</v>
       </c>
@@ -2429,7 +2454,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>52</v>
       </c>
@@ -2482,7 +2507,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
@@ -2533,7 +2558,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>72</v>
       </c>
@@ -2584,7 +2609,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>81</v>
       </c>
@@ -2747,7 +2772,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>107</v>
       </c>
@@ -2798,7 +2823,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>116</v>
       </c>
@@ -2849,7 +2874,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>126</v>
       </c>
@@ -2925,13 +2950,17 @@
       <c r="H14" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="I14" s="6"/>
+      <c r="I14" s="22" t="s">
+        <v>24</v>
+      </c>
       <c r="J14" s="4"/>
       <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
+      <c r="L14" s="22" t="s">
+        <v>511</v>
+      </c>
       <c r="M14" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>partly</v>
+        <v>correct</v>
       </c>
       <c r="N14" s="7" t="str">
         <f t="shared" si="1"/>
@@ -2953,7 +2982,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>144</v>
       </c>
@@ -3029,10 +3058,14 @@
       <c r="H16" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="I16" s="6"/>
+      <c r="I16" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="J16" s="4"/>
       <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
+      <c r="L16" s="22" t="s">
+        <v>505</v>
+      </c>
       <c r="M16" s="7" t="str">
         <f t="shared" si="0"/>
         <v>correct</v>
@@ -3044,7 +3077,7 @@
       <c r="O16" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="P16" s="4" t="s">
+      <c r="P16" s="23" t="s">
         <v>159</v>
       </c>
       <c r="Q16" s="4" t="s">
@@ -3057,7 +3090,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>163</v>
       </c>
@@ -3108,7 +3141,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>172</v>
       </c>
@@ -3184,10 +3217,14 @@
       <c r="H19" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="I19" s="6"/>
+      <c r="I19" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="J19" s="4"/>
       <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
+      <c r="L19" s="22" t="s">
+        <v>506</v>
+      </c>
       <c r="M19" s="7" t="str">
         <f t="shared" si="0"/>
         <v>correct</v>
@@ -3212,7 +3249,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>190</v>
       </c>
@@ -3263,7 +3300,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>199</v>
       </c>
@@ -3314,7 +3351,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>209</v>
       </c>
@@ -3365,7 +3402,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>220</v>
       </c>
@@ -3416,7 +3453,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>229</v>
       </c>
@@ -3492,16 +3529,22 @@
       <c r="H25" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="I25" s="6"/>
+      <c r="I25" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="J25" s="4"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6"/>
+      <c r="K25" s="22" t="s">
+        <v>508</v>
+      </c>
+      <c r="L25" s="22" t="s">
+        <v>507</v>
+      </c>
       <c r="M25" s="7" t="str">
         <f t="shared" si="0"/>
         <v>correct</v>
       </c>
       <c r="N25" s="7" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(K25="",J25&amp;"",IF(K25="no","",K25))</f>
         <v/>
       </c>
       <c r="O25" s="4" t="s">
@@ -3520,7 +3563,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>245</v>
       </c>
@@ -3571,7 +3614,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>254</v>
       </c>
@@ -3622,7 +3665,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>263</v>
       </c>
@@ -3673,7 +3716,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>272</v>
       </c>
@@ -3724,7 +3767,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>280</v>
       </c>
@@ -3775,7 +3818,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>290</v>
       </c>
@@ -3826,7 +3869,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>298</v>
       </c>
@@ -3877,7 +3920,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>307</v>
       </c>
@@ -3928,7 +3971,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>316</v>
       </c>
@@ -3979,7 +4022,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>325</v>
       </c>
@@ -4030,7 +4073,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>334</v>
       </c>
@@ -4081,7 +4124,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>343</v>
       </c>
@@ -4132,7 +4175,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>352</v>
       </c>
@@ -4183,7 +4226,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>362</v>
       </c>
@@ -4236,7 +4279,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>372</v>
       </c>
@@ -4287,7 +4330,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>381</v>
       </c>
@@ -4340,7 +4383,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>390</v>
       </c>
@@ -4391,7 +4434,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>399</v>
       </c>
@@ -4442,7 +4485,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>408</v>
       </c>
@@ -4520,10 +4563,14 @@
       <c r="H45" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="I45" s="6"/>
+      <c r="I45" s="6" t="s">
+        <v>92</v>
+      </c>
       <c r="J45" s="4"/>
       <c r="K45" s="6"/>
-      <c r="L45" s="6"/>
+      <c r="L45" s="22" t="s">
+        <v>509</v>
+      </c>
       <c r="M45" s="7" t="str">
         <f t="shared" si="2"/>
         <v>partly</v>
@@ -4548,7 +4595,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>426</v>
       </c>
@@ -4597,7 +4644,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>437</v>
       </c>
@@ -4646,7 +4693,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>444</v>
       </c>
@@ -4695,7 +4742,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>451</v>
       </c>
@@ -4744,7 +4791,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>457</v>
       </c>
@@ -4767,10 +4814,14 @@
       <c r="H50" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="I50" s="6"/>
+      <c r="I50" s="6" t="s">
+        <v>440</v>
+      </c>
       <c r="J50" s="4"/>
       <c r="K50" s="6"/>
-      <c r="L50" s="6"/>
+      <c r="L50" s="22" t="s">
+        <v>510</v>
+      </c>
       <c r="M50" s="7" t="str">
         <f t="shared" si="2"/>
         <v>answered beside the point</v>
@@ -4793,7 +4844,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:19" ht="150" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>463</v>
       </c>
@@ -4847,14 +4898,20 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S51" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:S51" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="M2:M51">
     <cfRule type="expression" dxfId="0" priority="2">
       <formula>AND(I2&lt;&gt;"",I2&lt;&gt;G2)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="K2:K51" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="K2:K51 L25" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"yes,no"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4940,7 +4997,7 @@
       </c>
       <c r="C5" s="12">
         <f>COUNTIFS(Review!$M$2:$M$51,$A5,Review!$B$2:$B$51,C$4)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5" s="12">
         <f>COUNTIFS(Review!$M$2:$M$51,$A5,Review!$B$2:$B$51,D$4)</f>
@@ -4960,7 +5017,7 @@
       </c>
       <c r="H5" s="13">
         <f t="shared" ref="H5:H12" si="0">SUM(B5:G5)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I5" s="12">
         <f>COUNTIF(Review!$G$2:$G$51,$A5)</f>
@@ -4968,7 +5025,7 @@
       </c>
       <c r="J5" s="12">
         <f t="shared" ref="J5:J12" si="1">H5-I5</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -4981,7 +5038,7 @@
       </c>
       <c r="C6" s="14">
         <f>COUNTIFS(Review!$M$2:$M$51,$A6,Review!$B$2:$B$51,C$4)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="14">
         <f>COUNTIFS(Review!$M$2:$M$51,$A6,Review!$B$2:$B$51,D$4)</f>
@@ -5001,7 +5058,7 @@
       </c>
       <c r="H6" s="15">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="14">
         <f>COUNTIF(Review!$G$2:$G$51,$A6)</f>
@@ -5009,7 +5066,7 @@
       </c>
       <c r="J6" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -5314,7 +5371,7 @@
       </c>
       <c r="B16" s="18">
         <f>SUM(B5:F5)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -5323,7 +5380,7 @@
       </c>
       <c r="B17" s="19">
         <f>IF(B15=0,0,B16/B15)</f>
-        <v>0.36363636363636365</v>
+        <v>0.38636363636363635</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -5350,7 +5407,7 @@
       </c>
       <c r="B20" s="18">
         <f>SUMPRODUCT((Review!$I$2:$I$51&lt;&gt;"")*(Review!$I$2:$I$51&lt;&gt;Review!$G$2:$G$51))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>